<commit_message>
Modifications 8 first files
</commit_message>
<xml_diff>
--- a/docs/pub_list/pub_list.xlsx
+++ b/docs/pub_list/pub_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\belli\OneDrive\Bureau\mywebsite\bbellier.com\pub_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5171D855-E3D7-4DE2-A21B-9C9A2E94AA0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8249252-8046-4330-8B78-073CCDA40F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -390,7 +390,13 @@
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="7" width="34.42578125" style="2" customWidth="1"/>
+    <col min="1" max="1" width="64.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="11" style="2" customWidth="1"/>
+    <col min="6" max="6" width="20.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="2" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
Modifications 9 first files
</commit_message>
<xml_diff>
--- a/docs/pub_list/pub_list.xlsx
+++ b/docs/pub_list/pub_list.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\belli\OneDrive\Bureau\mywebsite\bbellier.com\pub_list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8249252-8046-4330-8B78-073CCDA40F53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DA984B-6486-40AF-A354-7807DBA2D03E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1875" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Title</t>
   </si>
@@ -64,6 +64,30 @@
   </si>
   <si>
     <t>https://dx.doi.org/10.2139/ssrn.4717813</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>https://hdl.handle.net/10669/89985</t>
+  </si>
+  <si>
+    <t>Master</t>
+  </si>
+  <si>
+    <t>UCR</t>
+  </si>
+  <si>
+    <t>Efectos intergeneracionales de la exposición crónica a microplásticos de baja densidad en el zooplancton: el caso del copépodo Paracalanus parvus en el Golfo de Nicoya, Costa Rica</t>
+  </si>
+  <si>
+    <t>Universidad de Costa Rica, San José, Costa Rica</t>
+  </si>
+  <si>
+    <t>https://papers.ssrn.com/sol3/papers.cfm?abstract_id=4717813</t>
+  </si>
+  <si>
+    <t>pub_list/Bellier2023-UCR.pdf</t>
   </si>
 </sst>
 </file>
@@ -387,7 +411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="64.42578125" style="2" customWidth="1"/>
@@ -395,12 +419,12 @@
     <col min="3" max="3" width="15.85546875" style="2" customWidth="1"/>
     <col min="4" max="4" width="31.140625" style="2" customWidth="1"/>
     <col min="5" max="5" width="11" style="2" customWidth="1"/>
-    <col min="6" max="6" width="20.42578125" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="1"/>
+    <col min="6" max="7" width="20.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -420,10 +444,13 @@
         <v>8</v>
       </c>
       <c r="G1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="105" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
@@ -443,7 +470,33 @@
         <v>12</v>
       </c>
       <c r="G2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2023</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>